<commit_message>
Update package-lock.json and Vessels Log.xlsx
</commit_message>
<xml_diff>
--- a/backend/public/Vessels Log.xlsx
+++ b/backend/public/Vessels Log.xlsx
@@ -8676,7 +8676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I91"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.85546875" customWidth="1" min="1" max="1"/>
@@ -11511,96 +11511,6 @@
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>testtt</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>W/ MOORING BUOY</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>testtt</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>testtt</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>2025-11-02</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>10:07</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>10:12</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>testtt1</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>W/ MOORING BUOY</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>testtt1</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>testtt1</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>2025-11-03</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>10:59 AM</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>11:03 AM</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
improved analytics page and upcoming schedule widget automatically refreshes when adding a vessel.
</commit_message>
<xml_diff>
--- a/backend/public/Vessels Log.xlsx
+++ b/backend/public/Vessels Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raeve\Documents\school\anchorpoint-application\anchorpoint-application\backend\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8364C0F7-A4BE-49D2-B660-0219AEAEBF04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{660DE83B-5858-4E78-8FF3-DB7B79A7AA98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1291" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1240" uniqueCount="589">
   <si>
     <t>No.</t>
   </si>
@@ -1786,87 +1786,6 @@
   </si>
   <si>
     <t>October 16, 2025</t>
-  </si>
-  <si>
-    <t>test12</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>2025-10-29</t>
-  </si>
-  <si>
-    <t>04:09</t>
-  </si>
-  <si>
-    <t>Local</t>
-  </si>
-  <si>
-    <t>testing21</t>
-  </si>
-  <si>
-    <t>testing2</t>
-  </si>
-  <si>
-    <t>2025-10-30</t>
-  </si>
-  <si>
-    <t>08:02</t>
-  </si>
-  <si>
-    <t>Foreign</t>
-  </si>
-  <si>
-    <t>testing12</t>
-  </si>
-  <si>
-    <t>testing1</t>
-  </si>
-  <si>
-    <t>tset1</t>
-  </si>
-  <si>
-    <t>tset</t>
-  </si>
-  <si>
-    <t>2025-10-31</t>
-  </si>
-  <si>
-    <t>10:31</t>
-  </si>
-  <si>
-    <t>test21</t>
-  </si>
-  <si>
-    <t>test2</t>
-  </si>
-  <si>
-    <t>10:36</t>
-  </si>
-  <si>
-    <t>testtt</t>
-  </si>
-  <si>
-    <t>2025-11-02</t>
-  </si>
-  <si>
-    <t>10:07</t>
-  </si>
-  <si>
-    <t>10:12</t>
-  </si>
-  <si>
-    <t>testtt1</t>
-  </si>
-  <si>
-    <t>2025-11-03</t>
-  </si>
-  <si>
-    <t>10:59 AM</t>
-  </si>
-  <si>
-    <t>11:03 AM</t>
   </si>
   <si>
     <t>W/MOORING BOUY &amp; SHIFTING</t>
@@ -8666,7 +8585,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I91"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" customWidth="1"/>
@@ -9521,7 +9440,7 @@
         <v>64</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>615</v>
+        <v>588</v>
       </c>
       <c r="D37" s="11" t="s">
         <v>495</v>
@@ -10616,194 +10535,6 @@
       <c r="G84" s="23"/>
       <c r="H84" s="23"/>
       <c r="I84" s="23"/>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A85">
-        <v>84</v>
-      </c>
-      <c r="B85" t="s">
-        <v>588</v>
-      </c>
-      <c r="C85" t="s">
-        <v>429</v>
-      </c>
-      <c r="D85" t="s">
-        <v>589</v>
-      </c>
-      <c r="E85" t="s">
-        <v>589</v>
-      </c>
-      <c r="F85" t="s">
-        <v>590</v>
-      </c>
-      <c r="G85" t="s">
-        <v>591</v>
-      </c>
-      <c r="I85" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A86">
-        <v>86</v>
-      </c>
-      <c r="B86" t="s">
-        <v>593</v>
-      </c>
-      <c r="C86" t="s">
-        <v>384</v>
-      </c>
-      <c r="D86" t="s">
-        <v>594</v>
-      </c>
-      <c r="E86" t="s">
-        <v>594</v>
-      </c>
-      <c r="F86" t="s">
-        <v>595</v>
-      </c>
-      <c r="G86" t="s">
-        <v>596</v>
-      </c>
-      <c r="I86" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A87">
-        <v>87</v>
-      </c>
-      <c r="B87" t="s">
-        <v>598</v>
-      </c>
-      <c r="C87" t="s">
-        <v>429</v>
-      </c>
-      <c r="D87" t="s">
-        <v>599</v>
-      </c>
-      <c r="E87" t="s">
-        <v>599</v>
-      </c>
-      <c r="F87" t="s">
-        <v>590</v>
-      </c>
-      <c r="G87" t="s">
-        <v>596</v>
-      </c>
-      <c r="I87" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A88">
-        <v>88</v>
-      </c>
-      <c r="B88" t="s">
-        <v>600</v>
-      </c>
-      <c r="C88" t="s">
-        <v>429</v>
-      </c>
-      <c r="D88" t="s">
-        <v>601</v>
-      </c>
-      <c r="E88" t="s">
-        <v>601</v>
-      </c>
-      <c r="F88" t="s">
-        <v>602</v>
-      </c>
-      <c r="G88" t="s">
-        <v>603</v>
-      </c>
-      <c r="I88" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A89">
-        <v>88</v>
-      </c>
-      <c r="B89" t="s">
-        <v>604</v>
-      </c>
-      <c r="C89" t="s">
-        <v>429</v>
-      </c>
-      <c r="D89" t="s">
-        <v>605</v>
-      </c>
-      <c r="E89" t="s">
-        <v>605</v>
-      </c>
-      <c r="F89" t="s">
-        <v>595</v>
-      </c>
-      <c r="G89" t="s">
-        <v>606</v>
-      </c>
-      <c r="I89" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A90">
-        <v>89</v>
-      </c>
-      <c r="B90" t="s">
-        <v>607</v>
-      </c>
-      <c r="C90" t="s">
-        <v>429</v>
-      </c>
-      <c r="D90" t="s">
-        <v>607</v>
-      </c>
-      <c r="E90" t="s">
-        <v>607</v>
-      </c>
-      <c r="F90" t="s">
-        <v>608</v>
-      </c>
-      <c r="G90" t="s">
-        <v>609</v>
-      </c>
-      <c r="H90" t="s">
-        <v>610</v>
-      </c>
-      <c r="I90" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A91">
-        <v>90</v>
-      </c>
-      <c r="B91" t="s">
-        <v>611</v>
-      </c>
-      <c r="C91" t="s">
-        <v>429</v>
-      </c>
-      <c r="D91" t="s">
-        <v>611</v>
-      </c>
-      <c r="E91" t="s">
-        <v>611</v>
-      </c>
-      <c r="F91" t="s">
-        <v>612</v>
-      </c>
-      <c r="G91" t="s">
-        <v>613</v>
-      </c>
-      <c r="H91" t="s">
-        <v>614</v>
-      </c>
-      <c r="I91" t="s">
-        <v>592</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>